<commit_message>
Update extra fee hint, RatioFix balancing, and admin hardening
- shenbiao: 其他费用提示改为直白文案(进一法宁可多收也不少收)
- RatioFix: 配平器调整与兜底逻辑改进
- activation/admin/guoji: 安全加固与交互优化

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/演示/吧唧排表示例.xlsx
+++ b/演示/吧唧排表示例.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RenSheet\演示\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D915C04-8D2F-435E-9CD9-E59E3EFBF2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9BA7DE-0D51-4450-AF57-626D21EE24DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="21">
   <si>
     <t/>
   </si>
@@ -80,14 +80,6 @@
     <t>小丁</t>
   </si>
   <si>
-    <t>武道</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>麦</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>三途</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -97,6 +89,10 @@
   </si>
   <si>
     <t>立牌</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>武道</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -642,7 +638,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -662,24 +658,21 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
-      </c>
-      <c r="B3">
-        <v>28</v>
       </c>
       <c r="C3">
         <v>22</v>

</xml_diff>